<commit_message>
remove technical field names row from faculty/student import templates
- Delete the italic keys row (row 2) from both Arabic and English Excel templates
- Data now starts from row 2 instead of row 3
- Update import parser to no longer filter out key row
- Update photo extraction to skip row 1 only (was rows 1-2)
- Update data validation range, instruction text, and row number references
- Regenerate static template files in public/templates/
- Fix tests to match new row structure
</commit_message>
<xml_diff>
--- a/public/templates/faculty_members_template.xlsx
+++ b/public/templates/faculty_members_template.xlsx
@@ -1,59 +1,137 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011" filterPrivacy="true"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Members" sheetId="1" r:id="rId1"/>
-    <sheet name="تعليمات" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="الأعضاء" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
+  <si>
+    <t>الاسم الكامل</t>
+  </si>
+  <si>
+    <t>الوظيفة</t>
+  </si>
+  <si>
+    <t>القسم</t>
+  </si>
+  <si>
+    <t>تاريخ الميلاد (YYYY-MM-DD)</t>
+  </si>
+  <si>
+    <t>النوع</t>
+  </si>
+  <si>
+    <t>الرقم القومي</t>
+  </si>
+  <si>
+    <t>البريد الإلكتروني</t>
+  </si>
+  <si>
+    <t>رقم الهاتف</t>
+  </si>
+  <si>
+    <t>العنوان</t>
+  </si>
+  <si>
+    <t>المؤهل العلمي</t>
+  </si>
+  <si>
+    <t>التخصص</t>
+  </si>
+  <si>
+    <t>تاريخ التعيين (YYYY-MM-DD)</t>
+  </si>
+  <si>
+    <t>ملاحظات</t>
+  </si>
+  <si>
+    <t>رابط الصورة (اختياري)</t>
+  </si>
+  <si>
+    <t>صورة شخصية 4×6</t>
+  </si>
+  <si>
+    <t>أحمد محمد علي</t>
+  </si>
+  <si>
+    <t>دكتور</t>
+  </si>
+  <si>
+    <t>قسم علوم الحاسب</t>
+  </si>
+  <si>
+    <t>1985-05-12</t>
+  </si>
+  <si>
+    <t>male</t>
+  </si>
+  <si>
+    <t>29001011234567</t>
+  </si>
+  <si>
+    <t>ahmed@example.com</t>
+  </si>
+  <si>
+    <t>01000000000</t>
+  </si>
+  <si>
+    <t>القاهرة</t>
+  </si>
+  <si>
+    <t>دكتوراه</t>
+  </si>
+  <si>
+    <t>ذكاء اصطناعي</t>
+  </si>
+  <si>
+    <t>2020-09-01</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>https://example.com/photo.jpg</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF16A34A"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -61,18 +139,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF15803D"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -397,213 +495,121 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="18"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="28" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="24" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="32" customWidth="1"/>
+    <col min="15" max="15" width="18" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>الاسم الكامل</v>
-      </c>
-      <c r="B1" t="str">
-        <v>الوظيفة</v>
-      </c>
-      <c r="C1" t="str">
-        <v>القسم</v>
-      </c>
-      <c r="D1" t="str">
-        <v>تاريخ الميلاد (YYYY-MM-DD)</v>
-      </c>
-      <c r="E1" t="str">
-        <v>النوع</v>
-      </c>
-      <c r="F1" t="str">
-        <v>الرقم القومي</v>
-      </c>
-      <c r="G1" t="str">
-        <v>البريد الإلكتروني</v>
-      </c>
-      <c r="H1" t="str">
-        <v>رقم الهاتف</v>
-      </c>
-      <c r="I1" t="str">
-        <v>العنوان</v>
-      </c>
-      <c r="J1" t="str">
-        <v>المؤهل العلمي</v>
-      </c>
-      <c r="K1" t="str">
-        <v>التخصص</v>
-      </c>
-      <c r="L1" t="str">
-        <v>رابط الصورة (اختياري)</v>
-      </c>
-      <c r="M1" t="str">
-        <v>ملاحظات</v>
-      </c>
-      <c r="N1" t="str">
-        <v>صورة شخصية 4×6</v>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>full_name</v>
-      </c>
-      <c r="B2" t="str">
-        <v>role</v>
-      </c>
-      <c r="C2" t="str">
-        <v>department</v>
-      </c>
-      <c r="D2" t="str">
-        <v>date_of_birth</v>
-      </c>
-      <c r="E2" t="str">
-        <v>gender</v>
-      </c>
-      <c r="F2" t="str">
-        <v>national_id</v>
-      </c>
-      <c r="G2" t="str">
-        <v>email</v>
-      </c>
-      <c r="H2" t="str">
-        <v>phone</v>
-      </c>
-      <c r="I2" t="str">
-        <v>address</v>
-      </c>
-      <c r="J2" t="str">
-        <v>qualification</v>
-      </c>
-      <c r="K2" t="str">
-        <v>specialization</v>
-      </c>
-      <c r="L2" t="str">
-        <v>photo_url</v>
-      </c>
-      <c r="M2" t="str">
-        <v>notes</v>
-      </c>
-      <c r="N2" t="str">
-        <v>photo_image</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>أحمد محمد علي</v>
-      </c>
-      <c r="B3" t="str">
-        <v>دكتور</v>
-      </c>
-      <c r="C3" t="str">
-        <v>قسم علوم الحاسب</v>
-      </c>
-      <c r="D3" t="str">
-        <v>1985-05-12</v>
-      </c>
-      <c r="E3" t="str">
-        <v>male</v>
-      </c>
-      <c r="F3" t="str">
-        <v>29001011234567</v>
-      </c>
-      <c r="G3" t="str">
-        <v>ahmed@example.com</v>
-      </c>
-      <c r="H3" t="str">
-        <v>01000000000</v>
-      </c>
-      <c r="I3" t="str">
-        <v>القاهرة</v>
-      </c>
-      <c r="J3" t="str">
-        <v>دكتوراه</v>
-      </c>
-      <c r="K3" t="str">
-        <v>ذكاء اصطناعي</v>
-      </c>
-      <c r="L3" t="str">
-        <v>https://example.com/photo.jpg</v>
-      </c>
-      <c r="N3" t="str">
-        <v/>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A13"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>تعليمات تعبئة الملف:</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>1. لا تغيّر صف العناوين (الصف 1 و 2).</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2. ابدأ إدخال البيانات من الصف 3.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>3. الحقول المطلوبة: الاسم الكامل، الوظيفة، القسم.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>4. الوظيفة: اختر من القائمة المنسدلة.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>5. النوع: male أو female.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>6. التواريخ بصيغة YYYY-MM-DD.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>7. الرقم القومي والبريد والهاتف اختياري لكنه مفضل.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>9. رابط الصورة: أدخل رابط صورة العضو (اختياري). ارفع الصورة على أي خدمة استضافة ثم انسخ الرابط المباشر.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>الصور الشخصية</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>اختياري: أدرج صورة JPG أو PNG واحدة داخل خلية «صورة شخصية 4×6» في صف العضو. استخدم إدراج &gt; صور، ثم ضع الصورة داخل حدود الخلية.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Optional photo: insert one JPG or PNG into the member's 'صورة شخصية 4×6' cell. Use Insert &gt; Pictures and keep the image inside that cell.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A13"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>